<commit_message>
docs+data: update vay-chmeetings skill and lottery template
</commit_message>
<xml_diff>
--- a/middleware/data/2026-VAY-Lottery-Drawing_Team-Assignment(ALL-TEAM-SPORTS)_template.xlsx
+++ b/middleware/data/2026-VAY-Lottery-Drawing_Team-Assignment(ALL-TEAM-SPORTS)_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\MyPrj\vay\vaysf\middleware\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4798284F-1270-4767-B0A2-997B52206CCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B8380FC-2FC8-4094-A393-88EB61F7855A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="529" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -201,7 +201,7 @@
     <t>Team C</t>
   </si>
   <si>
-    <t>PHX</t>
+    <t>GEC</t>
   </si>
 </sst>
 </file>

</xml_diff>